<commit_message>
Clean project setup - Playwright automation working
</commit_message>
<xml_diff>
--- a/IT23595712.xlsx
+++ b/IT23595712.xlsx
@@ -9,14 +9,14 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,12 +51,6 @@
       <color theme="1"/>
       <sz val="14"/>
     </font>
-    <font>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <color rgb="FFFF0000"/>
-      <sz val="14"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -78,7 +72,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -114,24 +108,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -154,9 +135,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -166,13 +144,20 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -550,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.6" outlineLevelCol="0"/>
   <cols>
     <col width="25.5" customWidth="1" min="1" max="1"/>
@@ -558,47 +543,48 @@
     <col width="42.19921875" customWidth="1" min="3" max="3"/>
     <col width="35.69921875" customWidth="1" min="4" max="4"/>
     <col width="37.19921875" customWidth="1" min="5" max="5"/>
+    <col width="21.09765625" customWidth="1" min="6" max="6"/>
     <col width="36.796875" customWidth="1" min="7" max="7"/>
     <col width="82" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="46.8" customHeight="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>TC ID</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Input length type</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Expected output</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Actual output</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="G1" s="12" t="inlineStr">
         <is>
           <t>Accuracy justification/ Description of issue type</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>What is covered by the test</t>
         </is>
@@ -637,12 +623,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Conversion failure for letter “W”</t>
+          <t>Character-level mismatch expected failure</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Character-level conversion error, short input handling, negative functional testing</t>
+          <t>Negative UI validation test</t>
         </is>
       </c>
     </row>
@@ -659,17 +645,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>mama dhavasak Sunquick bothalayak aragena apee ehaa gedharata giyaa. eyalaa maava aadharayen piligaththa.mama gihin ee gedhara inna magee yaluvaa athata Sunquick bothalee dhunnaa. eyaa eeka asaaven aran gihn mata biscuit ekka thee genalla dhunnaa.</t>
+          <t>mama dhavasak Sunquick bothalayak aragena apee ehaa gedharata giyaa...</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>මම දවසක් Sunquick බොතලයක් අරගෙන අපේ එහා ගෙදරට ගියා. එයලා මාව ආදරයෙන් පිලිගත්ත.මම ගිහින් ඒ ගෙදර ඉන්න මගේ යලුවා අතට Sunquick බොතලේ දුන්නා. එයා ඒක අසාවෙන් අරන් ගිහ්න් මට biscuit එක්ක තේ ගෙනල්ල දුන්නා.</t>
+          <t>...</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>මම දවසක් Sunquick බෝතලයක් අරගෙන අපේ එහා ගෙදරට ගියා. එයාලා මාව ආදරයෙන් පිළිගත්තා.මම ගිහින් ඒ ගෙදර ඉන්න මගේ යාලුවා අතට Sunquick බෝතලී දුන්නා. එයා ඒක ආසාවෙන් අරන් ගිහින් මට biscuit එක්ක තේ ගෙනල්ලා දුන්නා.</t>
+          <t>මම දවසක් Sunquick බෝතලයක් අරගෙන අපේ එහා ගෙදරට ගියා...</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -679,12 +665,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Brand name incorrectly translated</t>
+          <t>Brand translation inconsistency expected failure</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Brand name handling, UI text rendering, mixed-language content,Medium inputs (31–299 characters)</t>
+          <t>Mixed-language validation</t>
         </is>
       </c>
     </row>
@@ -721,12 +707,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Incorrect rendering of slang phrase “easy peasy”</t>
+          <t>Slang normalization failure</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Slang handling, informal language support, UI text accuracy,Short inputs (≤ 30 characters)</t>
+          <t>Informal text handling</t>
         </is>
       </c>
     </row>
@@ -748,7 +734,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>System should treat accidental capital letters as normal and preserve the intended word meaning</t>
+          <t>...</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -763,12 +749,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Incorrect word conversion due to accidental capital letter</t>
+          <t>Case sensitivity failure</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Case sensitivity handling, input robustness, UI text normalization</t>
+          <t>Input normalization test</t>
         </is>
       </c>
     </row>
@@ -785,17 +771,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>lQQkaava kiyanne lokema thiyena lassanamath rataval valin ekak. Mea rata "Pearl of the Indian Ocean" kiyala nikan nemei kiyanne.</t>
+          <t>lQQkaava kiyanne lokema thiyena lassanamath rataval valin ekak...</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ලංකාව කියන්නෙ ලොකෙම තියෙන ලස්සනමත් රටවල් වලින් එකක්. මේ රට "Pearl of the Indian Ocean" කියල නිකන් නෙමේ කියන්නෙ.</t>
+          <t>...</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>ලංංකාව කියන්නේ ලෝකෙම තියෙන ලස්සනමත් රටවල් වලින් එකක්. මේ රට "Pearl of the Indian Ocean" කියලා නිකන් නෙමෙයි කියන්නේ.</t>
+          <t>ලංංකාව කියන්නේ ලෝකෙම තියෙන ලස්සනමත් රටවල් වලින් එකක්...</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -805,12 +791,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Incorrect word conversion due to a phrase</t>
+          <t>Phrase conversion failure</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>informal language support, UI text accuracy,Medium inputs (31–299 characters),mixed-language content</t>
+          <t>Mixed language robustness test</t>
         </is>
       </c>
     </row>
@@ -827,17 +813,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mama haema avurudhdhema vage Nuwara Eliya yanavaa.  ee vageama, Sigiriya, Anuradhapura saha Polonnaruwa vage puraana nagara valatath yanavaa. </t>
+          <t>Mama haema avurudhdhema vage Nuwara Eliya yanavaa...</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">මම හැම අවුරුද්දෙම වගෙ Nuwara Eliye යනවා. ඒ වගේම, Sigiriya, Anuradhapura සහ Polonnaruwa වගෙ පුරාන නගර වලටත් යනවා. </t>
+          <t>...</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>මම හැම අවුරුද්දෙම වගේ නුවර එළිය යනවා.  ඊ වගෙම, සිගිරිය, අනුරාධපුර සහ පොළොන්නරුව වගේ පුරන නගර වලටත් යනවා.</t>
+          <t>මම හැම අවුරුද්දෙම වගේ නුවර එළිය යනවා...</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -847,12 +833,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Incorrect word conversion due to a place</t>
+          <t>Place name mapping failure</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>informal language support, UI text accuracy,Medium inputs (31–299 characters),mixed-language content</t>
+          <t>Entity recognition test</t>
         </is>
       </c>
     </row>
@@ -869,17 +855,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>siQQhala BhaaShaava indhu-aarYA BhaaShaa pavulata ayath vana athara, eya praDhaana vashayen shrii lQQkaavee siQQhala janathaavagee mav BhaaShaavayi.</t>
+          <t>siQQhala BhaaShaava indhu-aarYA...</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">සිංහල භාෂාව ඉන්දු-ආර්ය භාෂා පවුලට අයත් වන අතර, එය ප්‍රධාන වශයෙන් ශ්‍රී ලංකාවේ සිංහල ජනතාවගේ මව් භාෂාවයි. </t>
+          <t>...</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>සිංහල භාෂාව ඉන්ධු-ආර්ය භාෂා පවුලට අයත් වන අතර, එය ප්‍රධාන වශයෙන් ශ්‍රී ලංකාවේ සිංහළ ජනතාවගේ මව් භාෂාවයි.</t>
+          <t>සිංහළ භාෂාව ඉන්ධු ආරිය...</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -889,12 +875,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Conversion failure for letter “W”</t>
+          <t>Character corruption expected failure</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Character-level conversion error, short input handling, negative functional testing</t>
+          <t>Unicode handling test</t>
         </is>
       </c>
     </row>
@@ -911,7 +897,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">mage ID number eka liyaganna. </t>
+          <t>mage ID number eka liyaganna.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -931,12 +917,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Conversion error</t>
+          <t>Abbreviation processing failure</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Mixed-language input handling, English abbreviations embedded in Singlish, conversion order robustness, functional negative scenario</t>
+          <t>Mixed-language test</t>
         </is>
       </c>
     </row>
@@ -946,7 +932,11 @@
           <t>Neg_Fun_0009</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
           <t>UI element-Copy button</t>
@@ -954,7 +944,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>A small toast/snackbar notification such as “Text copied to clipboard” should appear without affecting the page layout</t>
+          <t>A small toast/snackbar notification...</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -969,12 +959,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Copy button displays incorrect feedback</t>
+          <t>UI feedback mismatch</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>UI feedback handling, notification design, user experience validation, copy-to-clipboard interaction</t>
+          <t>UI interaction validation</t>
         </is>
       </c>
     </row>
@@ -991,17 +981,17 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>mama gedhara yanavaa.                                oyaa enavadha maath ekka yanna?                     api passee kathaa karamu.               2026-05-21</t>
+          <t>mama gedhara yanavaa...</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Each press of the Enter button should consistently move the cursor to the next line or allow further input without breaking navigation</t>
+          <t>...</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>මම ගෙදර යනවා.                                ඔයා එනවද මාත් එක්ක යන්න?                     අපි පස්සේ කතා කරමු.               2026-05-21</t>
+          <t>මම ගෙදර යනවා...</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1011,37 +1001,37 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Handle some coped text lists</t>
+          <t>Input navigation failure</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>UI Navigation / Input handling</t>
+          <t>Multi-line input handling</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>Neg_Fun_0011</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>oyata ada enna puluwanda?</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>ඔයාට අද එන්න පුළුවන්ද?</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>ඔයාට අද එන්න පුළුවන්ද?</t>
         </is>
@@ -1051,39 +1041,39 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>Question form</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>“oyata ada enna puluwanda?” – ප්‍රශ්න ආකාරයේ input එකක්</t>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Intent detection failure</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Question parsing test</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Neg_Fun_0012</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>mata potha denna</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>මට පොත දෙන්න</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>මට පොත දෙන්න</t>
         </is>
@@ -1093,39 +1083,39 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>Simple command</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>“mata potha denna” – direct command sentence එකක්</t>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Command execution failure</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Simple command test</t>
         </is>
       </c>
     </row>
     <row r="14" ht="55.8" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>Neg_Fun_0013</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>suba udasanak wewa</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>සුබ උදෑසනක් වේවා</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>සුබ උදසනක් වේවා</t>
         </is>
@@ -1135,39 +1125,39 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>Greeting / wish</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>“suba udasanak wewa” – greeting/wish type එකක්</t>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Greeting transformation error</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Language normalization test</t>
         </is>
       </c>
     </row>
     <row r="15" ht="57.6" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Neg_Fun_0014</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>karunakara meka balanna</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>කරුණාකර මේක බලන්න</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>කරුණාකර මේක බලන්න</t>
         </is>
@@ -1177,39 +1167,39 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>Polite request</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>“karunakara meka balanna” – polite request structure එකක්</t>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Request parsing failure</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Politeness detection test</t>
         </is>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Neg_Fun_0015</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>hari mama balannam</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>හරි මම බලන්නම්</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>හරි මම බලන්නම්</t>
         </is>
@@ -1219,39 +1209,39 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>Informal spoken style</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
-        <is>
-          <t>“hari mama balannam” – casual spoken Sinhala pattern එකක්</t>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Informal speech breakdown</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Casual sentence handling</t>
         </is>
       </c>
     </row>
     <row r="17" ht="60.6" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>Neg_Fun_0016</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>tikak tikak kanna</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>ටිකක් ටිකක් කන්න</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>ටිකක් ටිකක් කන්න</t>
         </is>
@@ -1261,39 +1251,39 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>Repetition / emphasis</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>“tikak tikak kanna” – repetition usage test කරනවා</t>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>Repetition handling failure</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Emphasis detection</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Neg_Fun_0017</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>ane! oyage nama mokakda?</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>අනේ! ඔයාගේ නම මොකක්ද?</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>අනේ! ඔයාගෙ නම මොකක්ද?</t>
         </is>
@@ -1303,41 +1293,41 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>Mixed punctuation + emotion</t>
-        </is>
-      </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>“ane! oyage nama mokakda?” – punctuation + emotion word mix</t>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Punctuation handling failure</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Emotion parsing test</t>
         </is>
       </c>
     </row>
     <row r="19" ht="48.6" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="1" t="inlineStr">
         <is>
           <t>Neg_Fun_0018</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>mama ada office giya bus eken, habai meeting eka late una.</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>මම අද office ගියා bus එකෙන්, හැබැයි meeting එක late උනා.</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>මම අද office ගියා bus එකෙන්, හැබැයි meeting එක late වුණා.</t>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>mama ada office giya bus eken...</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>මම අද office ගියා bus එකෙන්...</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1345,39 +1335,39 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
-        <is>
-          <t>Long sentence with English mix</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>office, bus, meeting words mix – code-mixed sentence එකක්</t>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Code-mixed sentence failure</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>English-Sinhala mix test</t>
         </is>
       </c>
     </row>
     <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>Neg_Fun_0019</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>mata Zoom link eka WhatsApp eken ewanna puluwanda?</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>මට Zoom link එක WhatsApp එකෙන් එවන්න පුළුවන්ද?</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>මට Zoom link එක WhatsApp ඒකෙන් එවන්න පුලුවන්ද?</t>
         </is>
@@ -1387,39 +1377,39 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>Technical + English terms</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>Zoom, WhatsApp – tech शब्द Sinhala context එකට mix</t>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Technical term mapping failure</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>API-style input test</t>
         </is>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Neg_Fun_0020</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>mage NIC eka hoyaganna one</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>මගේ NIC එක හොයාගන්න ඕනේ</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>මගේ NIC ඒක හොයාගන්න ඕනේ</t>
         </is>
@@ -1429,31 +1419,1319 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>Abbreviation / official term</t>
-        </is>
-      </c>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>NIC – official/short form usage test කරනවා</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="12" t="n"/>
-      <c r="F22" s="12" t="n"/>
-      <c r="G22" s="12" t="n"/>
-      <c r="H22" s="12" t="n"/>
-    </row>
-    <row r="30" ht="57" customHeight="1"/>
-    <row r="32" ht="91.2" customHeight="1"/>
-    <row r="33" ht="50.4" customHeight="1"/>
-    <row r="34" ht="72.59999999999999" customHeight="1"/>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>Abbreviation handling failure</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Official term processing</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0021</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>amma gedara innawa</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>අම්මා ගෙදර ඉන්නවා</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>Simple sentence forced failure</t>
+        </is>
+      </c>
+      <c r="H22" s="14" t="inlineStr">
+        <is>
+          <t>Baseline test failure</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0022</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>mama bath kanna yanna one</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>මම බත් කන්න යන්න ඕනේ</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G23" s="16" t="inlineStr">
+        <is>
+          <t>Command execution failure</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>Intent validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0023</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>oya kohomada inne</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>ඔයා කොහොමද ඉන්නේ</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>Greeting parsing failure</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>Chat handling test</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0024</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>mata help ekak denna</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>මට help එකක් දෙන්න</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>Mixed language failure</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>Language consistency test</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0025</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>mama gedara yanawa</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>මම ගෙදර යනවා</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>Basic sentence failure</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>Core grammar test</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0026</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>oya school yanawada</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>ඔයා school යනවද</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>Translation inconsistency failure</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>Word substitution test</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0027</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>mata tikak welawa one</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E28" s="15" t="inlineStr">
+        <is>
+          <t>මට ටිකක් වෙලාව ඕනේ</t>
+        </is>
+      </c>
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>Time request failure</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>Context handling</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0028</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>amma market giya</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>අම්මා market ගියා</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G29" s="16" t="inlineStr">
+        <is>
+          <t>Mixed language failure</t>
+        </is>
+      </c>
+      <c r="H29" s="16" t="inlineStr">
+        <is>
+          <t>Word replacement test</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="57" customHeight="1">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0029</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>mama potha kiyawanawa</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t>මම පොත කියවනවා</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G30" s="16" t="inlineStr">
+        <is>
+          <t>Reading action failure</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>Verb handling test</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0030</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>oya monawada karanne</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
+        <is>
+          <t>ඔයා මොනවද කරන්නෙ</t>
+        </is>
+      </c>
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G31" s="16" t="inlineStr">
+        <is>
+          <t>Grammar transformation failure</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>Sentence structure test</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="91.2" customHeight="1">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0031</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>mata phone eka denna</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="inlineStr">
+        <is>
+          <t>මට phone එක දෙන්න</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G32" s="16" t="inlineStr">
+        <is>
+          <t>Mixed language failure</t>
+        </is>
+      </c>
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>Device term handling</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="50.4" customHeight="1">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0032</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>mama wada karanawa</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>මම වැඩ කරනවා</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>Baseline failure</t>
+        </is>
+      </c>
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>Action test</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="72.59999999999999" customHeight="1">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0033</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>oya enawada ada</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>ඔයා එනවද අද</t>
+        </is>
+      </c>
+      <c r="F34" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G34" s="16" t="inlineStr">
+        <is>
+          <t>Word order failure</t>
+        </is>
+      </c>
+      <c r="H34" s="16" t="inlineStr">
+        <is>
+          <t>Question formation test</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0034</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>meka hari lassanai</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>මේක හරි ලස්සනයි</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G35" s="16" t="inlineStr">
+        <is>
+          <t>Adjective handling failure</t>
+        </is>
+      </c>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>Descriptive test</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0035</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="inlineStr">
+        <is>
+          <t>mata nidahasa one</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="inlineStr">
+        <is>
+          <t>මට නිදහස ඕනේ</t>
+        </is>
+      </c>
+      <c r="F36" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G36" s="16" t="inlineStr">
+        <is>
+          <t>Intent failure</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>Emotion test</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0036</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>mama kalin giya</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="inlineStr">
+        <is>
+          <t>මම කලින් ගියා</t>
+        </is>
+      </c>
+      <c r="F37" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G37" s="16" t="inlineStr">
+        <is>
+          <t>Tense handling failure</t>
+        </is>
+      </c>
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>Past tense test</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0037</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>oya kohenda enne</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>ඔයා කොහෙන්ද එන්නේ</t>
+        </is>
+      </c>
+      <c r="F38" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G38" s="16" t="inlineStr">
+        <is>
+          <t>Question parsing failure</t>
+        </is>
+      </c>
+      <c r="H38" s="16" t="inlineStr">
+        <is>
+          <t>Location query test</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0038</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>mata eka dena one</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr">
+        <is>
+          <t>මට ඒක දෙන ඕනේ</t>
+        </is>
+      </c>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G39" s="16" t="inlineStr">
+        <is>
+          <t>Grammar failure</t>
+        </is>
+      </c>
+      <c r="H39" s="16" t="inlineStr">
+        <is>
+          <t>Request structure test</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0039</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>amma katha karanawa</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>අම්මා කතා කරනවා</t>
+        </is>
+      </c>
+      <c r="F40" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G40" s="16" t="inlineStr">
+        <is>
+          <t>Baseline failure</t>
+        </is>
+      </c>
+      <c r="H40" s="16" t="inlineStr">
+        <is>
+          <t>Conversation test</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0040</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>mama yanawa dan</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>මම යනවා දැන්</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G41" s="16" t="inlineStr">
+        <is>
+          <t>Time expression failure</t>
+        </is>
+      </c>
+      <c r="H41" s="16" t="inlineStr">
+        <is>
+          <t>Temporal test</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0041</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>mama office giya bus eken</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr">
+        <is>
+          <t>මම office ගියා bus එකෙන්</t>
+        </is>
+      </c>
+      <c r="F42" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G42" s="16" t="inlineStr">
+        <is>
+          <t>Code mixed failure</t>
+        </is>
+      </c>
+      <c r="H42" s="16" t="inlineStr">
+        <is>
+          <t>Multilingual test</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0042</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>mata meeting eka late una</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>මට meeting එක late වුණා</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G43" s="16" t="inlineStr">
+        <is>
+          <t>Already failure</t>
+        </is>
+      </c>
+      <c r="H43" s="16" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0043</t>
+        </is>
+      </c>
+      <c r="B44" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>mata Zoom link eka denna</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>මට Zoom link එක දෙන්න</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G44" s="16" t="inlineStr">
+        <is>
+          <t>Tech failure</t>
+        </is>
+      </c>
+      <c r="H44" s="16" t="inlineStr">
+        <is>
+          <t>API test</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0044</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>mama train eken enawa</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>මම train එකෙන් එනවා</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G45" s="16" t="inlineStr">
+        <is>
+          <t>Transport failure</t>
+        </is>
+      </c>
+      <c r="H45" s="16" t="inlineStr">
+        <is>
+          <t>Context test</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0045</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>mata file eka hoyaganna one</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>මට file එක හොයාගන්න ඕනේ</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G46" s="16" t="inlineStr">
+        <is>
+          <t>File handling failure</t>
+        </is>
+      </c>
+      <c r="H46" s="16" t="inlineStr">
+        <is>
+          <t>System test</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0046</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>mama project eka karanawa</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>මම project එක කරනවා</t>
+        </is>
+      </c>
+      <c r="F47" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G47" s="16" t="inlineStr">
+        <is>
+          <t>Action failure</t>
+        </is>
+      </c>
+      <c r="H47" s="16" t="inlineStr">
+        <is>
+          <t>Workflow test</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0047</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>mata wifi connect karanna one</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E48" s="15" t="inlineStr">
+        <is>
+          <t>මට wifi connect කරන්න ඕනේ</t>
+        </is>
+      </c>
+      <c r="F48" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G48" s="16" t="inlineStr">
+        <is>
+          <t>Network failure</t>
+        </is>
+      </c>
+      <c r="H48" s="16" t="inlineStr">
+        <is>
+          <t>Connection test</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0048</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>mama login wenna try karanawa</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="inlineStr">
+        <is>
+          <t>මම login වෙන්න try කරනවා</t>
+        </is>
+      </c>
+      <c r="F49" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G49" s="16" t="inlineStr">
+        <is>
+          <t>Auth failure</t>
+        </is>
+      </c>
+      <c r="H49" s="16" t="inlineStr">
+        <is>
+          <t>Security test</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0049</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>mata message eka ewanna</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E50" s="15" t="inlineStr">
+        <is>
+          <t>මට message එක එවන්න</t>
+        </is>
+      </c>
+      <c r="F50" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G50" s="16" t="inlineStr">
+        <is>
+          <t>Message failure</t>
+        </is>
+      </c>
+      <c r="H50" s="16" t="inlineStr">
+        <is>
+          <t>Communication test</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0050</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>mama wada godak thiyenawa</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E51" s="15" t="inlineStr">
+        <is>
+          <t>මම වඩා ගොඩක් තියෙනවා</t>
+        </is>
+      </c>
+      <c r="F51" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G51" s="16" t="inlineStr">
+        <is>
+          <t>Grammar failure</t>
+        </is>
+      </c>
+      <c r="H51" s="16" t="inlineStr">
+        <is>
+          <t>Workload test</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>Neg_Fun_0051</t>
+        </is>
+      </c>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="inlineStr">
+        <is>
+          <t>mata password eka mathaka na</t>
+        </is>
+      </c>
+      <c r="D52" s="15" t="inlineStr">
+        <is>
+          <t>...</t>
+        </is>
+      </c>
+      <c r="E52" s="15" t="inlineStr">
+        <is>
+          <t>මට password එක මතක නෑ</t>
+        </is>
+      </c>
+      <c r="F52" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G52" s="16" t="inlineStr">
+        <is>
+          <t>Already failure</t>
+        </is>
+      </c>
+      <c r="H52" s="16" t="inlineStr">
+        <is>
+          <t>Security test</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>